<commit_message>
av01: fix boss not scrolling down
</commit_message>
<xml_diff>
--- a/av01/spawn_config.xlsx
+++ b/av01/spawn_config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Git\av01\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{010BAAEC-78D4-4DEE-A4D8-6D901E504472}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A471B79F-3197-4FDE-874C-C80D971095E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1290" yWindow="1305" windowWidth="28695" windowHeight="15240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="15">
   <si>
     <t>tick</t>
   </si>
@@ -68,19 +68,17 @@
     <t>main_0</t>
   </si>
   <si>
-    <t>main_1</t>
-  </si>
-  <si>
     <t>barrel</t>
   </si>
   <si>
     <t>center</t>
   </si>
   <si>
-    <t>main_2</t>
+    <t>boss</t>
   </si>
   <si>
-    <t>boss</t>
+    <t>main_2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -464,7 +462,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F93"/>
+  <dimension ref="A1:G92"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="6.875" customWidth="1"/>
@@ -474,7 +472,7 @@
     <col min="6" max="6" width="12.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -494,7 +492,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A2">
         <v>1</v>
       </c>
@@ -508,7 +506,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A3">
         <v>1</v>
       </c>
@@ -522,7 +520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A4">
         <v>2</v>
       </c>
@@ -536,7 +534,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A5">
         <v>2</v>
       </c>
@@ -550,7 +548,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A6">
         <v>3</v>
       </c>
@@ -564,7 +562,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A7">
         <v>3</v>
       </c>
@@ -578,7 +576,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A8">
         <v>3</v>
       </c>
@@ -592,9 +590,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B9" t="s">
         <v>9</v>
@@ -606,9 +604,9 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A10">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B10" t="s">
         <v>6</v>
@@ -619,10 +617,14 @@
       <c r="D10">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G10">
+        <f>A10+2</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A11">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B11" t="s">
         <v>6</v>
@@ -633,10 +635,14 @@
       <c r="D11">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G11">
+        <f t="shared" ref="G11:G70" si="0">A11+2</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A12">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B12" t="s">
         <v>6</v>
@@ -647,10 +653,14 @@
       <c r="D12">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G12">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A13">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B13" t="s">
         <v>8</v>
@@ -661,10 +671,14 @@
       <c r="D13">
         <v>10</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G13">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A14">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B14" t="s">
         <v>6</v>
@@ -675,10 +689,14 @@
       <c r="D14">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G14">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A15">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B15" t="s">
         <v>6</v>
@@ -689,10 +707,14 @@
       <c r="D15">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G15">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A16">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B16" t="s">
         <v>6</v>
@@ -703,10 +725,14 @@
       <c r="D16">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G16">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A17">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B17" t="s">
         <v>6</v>
@@ -717,10 +743,14 @@
       <c r="D17">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G17">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A18">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B18" t="s">
         <v>6</v>
@@ -731,10 +761,14 @@
       <c r="D18">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G18">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A19">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B19" t="s">
         <v>6</v>
@@ -745,10 +779,14 @@
       <c r="D19">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G19">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A20">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B20" t="s">
         <v>6</v>
@@ -759,10 +797,14 @@
       <c r="D20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G20">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A21">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B21" t="s">
         <v>6</v>
@@ -773,10 +815,14 @@
       <c r="D21">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G21">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A22">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B22" t="s">
         <v>6</v>
@@ -787,10 +833,14 @@
       <c r="D22">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G22">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A23">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B23" t="s">
         <v>6</v>
@@ -801,10 +851,14 @@
       <c r="D23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G23">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A24">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B24" t="s">
         <v>6</v>
@@ -815,10 +869,14 @@
       <c r="D24">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G24">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A25">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B25" t="s">
         <v>8</v>
@@ -829,10 +887,14 @@
       <c r="D25">
         <v>10</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G25">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A26">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B26" t="s">
         <v>6</v>
@@ -843,24 +905,32 @@
       <c r="D26">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G26">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A27">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B27" t="s">
         <v>9</v>
       </c>
       <c r="C27" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E27">
         <v>-15</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G27">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A28">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B28" t="s">
         <v>6</v>
@@ -871,16 +941,20 @@
       <c r="D28">
         <v>1</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G28">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A29">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B29" t="s">
+        <v>11</v>
+      </c>
+      <c r="C29" t="s">
         <v>12</v>
-      </c>
-      <c r="C29" t="s">
-        <v>13</v>
       </c>
       <c r="D29">
         <v>30</v>
@@ -888,10 +962,14 @@
       <c r="F29">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G29">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A30">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B30" t="s">
         <v>6</v>
@@ -902,10 +980,14 @@
       <c r="D30">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G30">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A31">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B31" t="s">
         <v>6</v>
@@ -916,10 +998,14 @@
       <c r="D31">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G31">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A32">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B32" t="s">
         <v>6</v>
@@ -930,10 +1016,14 @@
       <c r="D32">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G32">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A33">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B33" t="s">
         <v>6</v>
@@ -944,10 +1034,14 @@
       <c r="D33">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G33">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A34">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B34" t="s">
         <v>6</v>
@@ -958,10 +1052,14 @@
       <c r="D34">
         <v>1</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G34">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A35">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B35" t="s">
         <v>6</v>
@@ -972,10 +1070,14 @@
       <c r="D35">
         <v>1</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G35">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A36">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B36" t="s">
         <v>6</v>
@@ -986,10 +1088,14 @@
       <c r="D36">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G36">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A37">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B37" t="s">
         <v>8</v>
@@ -1000,10 +1106,14 @@
       <c r="D37">
         <v>10</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G37">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A38">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B38" t="s">
         <v>6</v>
@@ -1014,10 +1124,14 @@
       <c r="D38">
         <v>1</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G38">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A39">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B39" t="s">
         <v>6</v>
@@ -1028,10 +1142,14 @@
       <c r="D39">
         <v>1</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G39">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A40">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B40" t="s">
         <v>6</v>
@@ -1042,10 +1160,14 @@
       <c r="D40">
         <v>1</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G40">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A41">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B41" t="s">
         <v>6</v>
@@ -1056,10 +1178,14 @@
       <c r="D41">
         <v>1</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G41">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A42">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B42" t="s">
         <v>6</v>
@@ -1070,10 +1196,14 @@
       <c r="D42">
         <v>1</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G42">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A43">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B43" t="s">
         <v>6</v>
@@ -1084,24 +1214,32 @@
       <c r="D43">
         <v>1</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G43">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A44">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B44" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C44" t="s">
-        <v>14</v>
-      </c>
-      <c r="E44">
-        <v>-75</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+        <v>7</v>
+      </c>
+      <c r="D44">
+        <v>1</v>
+      </c>
+      <c r="G44">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A45">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B45" t="s">
         <v>6</v>
@@ -1112,10 +1250,14 @@
       <c r="D45">
         <v>1</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G45">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A46">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B46" t="s">
         <v>6</v>
@@ -1126,38 +1268,50 @@
       <c r="D46">
         <v>1</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G46">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A47">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B47" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C47" t="s">
         <v>7</v>
       </c>
       <c r="D47">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+        <v>10</v>
+      </c>
+      <c r="G47">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A48">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B48" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C48" t="s">
         <v>7</v>
       </c>
       <c r="D48">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+        <v>1</v>
+      </c>
+      <c r="G48">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A49">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B49" t="s">
         <v>6</v>
@@ -1168,10 +1322,14 @@
       <c r="D49">
         <v>1</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G49">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A50">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B50" t="s">
         <v>6</v>
@@ -1182,10 +1340,14 @@
       <c r="D50">
         <v>1</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G50">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A51">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B51" t="s">
         <v>6</v>
@@ -1196,10 +1358,14 @@
       <c r="D51">
         <v>1</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G51">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A52">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B52" t="s">
         <v>6</v>
@@ -1210,10 +1376,14 @@
       <c r="D52">
         <v>1</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G52">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A53">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B53" t="s">
         <v>6</v>
@@ -1224,10 +1394,14 @@
       <c r="D53">
         <v>1</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G53">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A54">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B54" t="s">
         <v>6</v>
@@ -1238,257 +1412,312 @@
       <c r="D54">
         <v>1</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="G54">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A55">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B55" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C55" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D55">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+        <v>120</v>
+      </c>
+      <c r="F55">
+        <v>2</v>
+      </c>
+      <c r="G55">
+        <f t="shared" si="0"/>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A56">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B56" t="s">
+        <v>6</v>
+      </c>
+      <c r="C56" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56">
+        <v>1</v>
+      </c>
+      <c r="G56">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A57">
+        <v>32</v>
+      </c>
+      <c r="B57" t="s">
+        <v>6</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57">
+        <v>1</v>
+      </c>
+      <c r="G57">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A58">
+        <v>33</v>
+      </c>
+      <c r="B58" t="s">
+        <v>6</v>
+      </c>
+      <c r="C58" t="s">
+        <v>7</v>
+      </c>
+      <c r="D58">
+        <v>1</v>
+      </c>
+      <c r="G58">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A59">
+        <v>33</v>
+      </c>
+      <c r="B59" t="s">
+        <v>6</v>
+      </c>
+      <c r="C59" t="s">
+        <v>7</v>
+      </c>
+      <c r="D59">
+        <v>1</v>
+      </c>
+      <c r="G59">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A60">
+        <v>34</v>
+      </c>
+      <c r="B60" t="s">
+        <v>6</v>
+      </c>
+      <c r="C60" t="s">
+        <v>7</v>
+      </c>
+      <c r="D60">
+        <v>1</v>
+      </c>
+      <c r="G60">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A61">
+        <v>34</v>
+      </c>
+      <c r="B61" t="s">
+        <v>6</v>
+      </c>
+      <c r="C61" t="s">
+        <v>7</v>
+      </c>
+      <c r="D61">
+        <v>1</v>
+      </c>
+      <c r="G61">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A62">
+        <v>34</v>
+      </c>
+      <c r="B62" t="s">
+        <v>6</v>
+      </c>
+      <c r="C62" t="s">
+        <v>7</v>
+      </c>
+      <c r="D62">
+        <v>1</v>
+      </c>
+      <c r="G62">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A63">
+        <v>35</v>
+      </c>
+      <c r="B63" t="s">
+        <v>6</v>
+      </c>
+      <c r="C63" t="s">
+        <v>7</v>
+      </c>
+      <c r="D63">
+        <v>1</v>
+      </c>
+      <c r="G63">
+        <f t="shared" si="0"/>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A64">
+        <v>35</v>
+      </c>
+      <c r="B64" t="s">
+        <v>6</v>
+      </c>
+      <c r="C64" t="s">
+        <v>7</v>
+      </c>
+      <c r="D64">
+        <v>1</v>
+      </c>
+      <c r="G64">
+        <f t="shared" si="0"/>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A65">
+        <v>36</v>
+      </c>
+      <c r="B65" t="s">
+        <v>6</v>
+      </c>
+      <c r="C65" t="s">
+        <v>7</v>
+      </c>
+      <c r="D65">
+        <v>1</v>
+      </c>
+      <c r="G65">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A66">
+        <v>36</v>
+      </c>
+      <c r="B66" t="s">
+        <v>6</v>
+      </c>
+      <c r="C66" t="s">
+        <v>7</v>
+      </c>
+      <c r="D66">
+        <v>1</v>
+      </c>
+      <c r="G66">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A67">
+        <v>37</v>
+      </c>
+      <c r="B67" t="s">
+        <v>6</v>
+      </c>
+      <c r="C67" t="s">
+        <v>7</v>
+      </c>
+      <c r="D67">
+        <v>1</v>
+      </c>
+      <c r="G67">
+        <f t="shared" si="0"/>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A68">
+        <v>37</v>
+      </c>
+      <c r="B68" t="s">
+        <v>6</v>
+      </c>
+      <c r="C68" t="s">
+        <v>7</v>
+      </c>
+      <c r="D68">
+        <v>1</v>
+      </c>
+      <c r="G68">
+        <f t="shared" si="0"/>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A69">
+        <v>37</v>
+      </c>
+      <c r="B69" t="s">
+        <v>6</v>
+      </c>
+      <c r="C69" t="s">
+        <v>7</v>
+      </c>
+      <c r="D69">
+        <v>1</v>
+      </c>
+      <c r="G69">
+        <f t="shared" si="0"/>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A70">
+        <v>38</v>
+      </c>
+      <c r="B70" t="s">
+        <v>13</v>
+      </c>
+      <c r="C70" t="s">
         <v>12</v>
       </c>
-      <c r="C56" t="s">
-        <v>13</v>
-      </c>
-      <c r="D56">
-        <v>120</v>
-      </c>
-      <c r="F56">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A57">
-        <v>30</v>
-      </c>
-      <c r="B57" t="s">
-        <v>6</v>
-      </c>
-      <c r="C57" t="s">
-        <v>7</v>
-      </c>
-      <c r="D57">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A58">
-        <v>30</v>
-      </c>
-      <c r="B58" t="s">
-        <v>6</v>
-      </c>
-      <c r="C58" t="s">
-        <v>7</v>
-      </c>
-      <c r="D58">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A59">
-        <v>31</v>
-      </c>
-      <c r="B59" t="s">
-        <v>6</v>
-      </c>
-      <c r="C59" t="s">
-        <v>7</v>
-      </c>
-      <c r="D59">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A60">
-        <v>31</v>
-      </c>
-      <c r="B60" t="s">
-        <v>6</v>
-      </c>
-      <c r="C60" t="s">
-        <v>7</v>
-      </c>
-      <c r="D60">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A61">
-        <v>32</v>
-      </c>
-      <c r="B61" t="s">
-        <v>6</v>
-      </c>
-      <c r="C61" t="s">
-        <v>7</v>
-      </c>
-      <c r="D61">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A62">
-        <v>32</v>
-      </c>
-      <c r="B62" t="s">
-        <v>6</v>
-      </c>
-      <c r="C62" t="s">
-        <v>7</v>
-      </c>
-      <c r="D62">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A63">
-        <v>32</v>
-      </c>
-      <c r="B63" t="s">
-        <v>6</v>
-      </c>
-      <c r="C63" t="s">
-        <v>7</v>
-      </c>
-      <c r="D63">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A64">
-        <v>33</v>
-      </c>
-      <c r="B64" t="s">
-        <v>6</v>
-      </c>
-      <c r="C64" t="s">
-        <v>7</v>
-      </c>
-      <c r="D64">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A65">
-        <v>33</v>
-      </c>
-      <c r="B65" t="s">
-        <v>6</v>
-      </c>
-      <c r="C65" t="s">
-        <v>7</v>
-      </c>
-      <c r="D65">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A66">
-        <v>34</v>
-      </c>
-      <c r="B66" t="s">
-        <v>6</v>
-      </c>
-      <c r="C66" t="s">
-        <v>7</v>
-      </c>
-      <c r="D66">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A67">
-        <v>34</v>
-      </c>
-      <c r="B67" t="s">
-        <v>6</v>
-      </c>
-      <c r="C67" t="s">
-        <v>7</v>
-      </c>
-      <c r="D67">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A68">
-        <v>35</v>
-      </c>
-      <c r="B68" t="s">
-        <v>6</v>
-      </c>
-      <c r="C68" t="s">
-        <v>7</v>
-      </c>
-      <c r="D68">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A69">
-        <v>35</v>
-      </c>
-      <c r="B69" t="s">
-        <v>6</v>
-      </c>
-      <c r="C69" t="s">
-        <v>7</v>
-      </c>
-      <c r="D69">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A70">
-        <v>35</v>
-      </c>
-      <c r="B70" t="s">
-        <v>6</v>
-      </c>
-      <c r="C70" t="s">
-        <v>7</v>
-      </c>
       <c r="D70">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A71">
-        <v>36</v>
-      </c>
-      <c r="B71" t="s">
-        <v>15</v>
-      </c>
-      <c r="C71" t="s">
-        <v>13</v>
-      </c>
-      <c r="D71">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" ht="14.25" x14ac:dyDescent="0.15"/>
-    <row r="73" spans="1:4" ht="14.25" x14ac:dyDescent="0.15"/>
-    <row r="74" spans="1:4" ht="14.25" x14ac:dyDescent="0.15"/>
-    <row r="75" spans="1:4" ht="14.25" x14ac:dyDescent="0.15"/>
-    <row r="76" spans="1:4" ht="14.25" x14ac:dyDescent="0.15"/>
-    <row r="77" spans="1:4" ht="14.25" x14ac:dyDescent="0.15"/>
-    <row r="78" spans="1:4" ht="14.25" x14ac:dyDescent="0.15"/>
-    <row r="79" spans="1:4" ht="14.25" x14ac:dyDescent="0.15"/>
-    <row r="80" spans="1:4" ht="14.25" x14ac:dyDescent="0.15"/>
+        <v>1000</v>
+      </c>
+      <c r="G70">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" ht="14.25" x14ac:dyDescent="0.15"/>
+    <row r="72" spans="1:7" ht="14.25" x14ac:dyDescent="0.15"/>
+    <row r="73" spans="1:7" ht="14.25" x14ac:dyDescent="0.15"/>
+    <row r="74" spans="1:7" ht="14.25" x14ac:dyDescent="0.15"/>
+    <row r="75" spans="1:7" ht="14.25" x14ac:dyDescent="0.15"/>
+    <row r="76" spans="1:7" ht="14.25" x14ac:dyDescent="0.15"/>
+    <row r="77" spans="1:7" ht="14.25" x14ac:dyDescent="0.15"/>
+    <row r="78" spans="1:7" ht="14.25" x14ac:dyDescent="0.15"/>
+    <row r="79" spans="1:7" ht="14.25" x14ac:dyDescent="0.15"/>
+    <row r="80" spans="1:7" ht="14.25" x14ac:dyDescent="0.15"/>
     <row r="81" ht="14.25" x14ac:dyDescent="0.15"/>
     <row r="82" ht="14.25" x14ac:dyDescent="0.15"/>
     <row r="83" ht="14.25" x14ac:dyDescent="0.15"/>
@@ -1501,13 +1730,12 @@
     <row r="90" ht="14.25" x14ac:dyDescent="0.15"/>
     <row r="91" ht="14.25" x14ac:dyDescent="0.15"/>
     <row r="92" ht="14.25" x14ac:dyDescent="0.15"/>
-    <row r="93" ht="14.25" x14ac:dyDescent="0.15"/>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A10:F12 A1:F8 A14:F23 B13:F13 B29:F37 B39:F43 B45:F55 B57:F71 B27:F27 B25:F25" numberStoredAsText="1"/>
+    <ignoredError sqref="B10:F12 A1:F8 B14:F23 B13:F13 B29:F37 B39:F43 B44:F54 B56:F69 B27 B25:F25 B70:C70 E70:F70 D27:F27" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
av01: instant first spawn, homing center-hit
</commit_message>
<xml_diff>
--- a/av01/spawn_config.xlsx
+++ b/av01/spawn_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Git\av01\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A471B79F-3197-4FDE-874C-C80D971095E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D7E2A08-1FE7-4BFD-A2A6-9471ADE000FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1290" yWindow="1305" windowWidth="28695" windowHeight="15240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Spawns" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="15">
   <si>
     <t>tick</t>
   </si>
@@ -462,7 +462,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G92"/>
+  <dimension ref="A1:F99"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="6.875" customWidth="1"/>
@@ -472,7 +472,7 @@
     <col min="6" max="6" width="12.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -492,7 +492,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A2">
         <v>1</v>
       </c>
@@ -506,7 +506,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A3">
         <v>1</v>
       </c>
@@ -520,7 +520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A4">
         <v>2</v>
       </c>
@@ -534,7 +534,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A5">
         <v>2</v>
       </c>
@@ -548,7 +548,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A6">
         <v>3</v>
       </c>
@@ -562,7 +562,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A7">
         <v>3</v>
       </c>
@@ -576,7 +576,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A8">
         <v>3</v>
       </c>
@@ -590,7 +590,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A9">
         <v>5</v>
       </c>
@@ -601,10 +601,10 @@
         <v>10</v>
       </c>
       <c r="E9">
-        <v>-3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+        <v>-15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A10">
         <v>7</v>
       </c>
@@ -617,12 +617,8 @@
       <c r="D10">
         <v>1</v>
       </c>
-      <c r="G10">
-        <f>A10+2</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="11" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A11">
         <v>7</v>
       </c>
@@ -635,12 +631,8 @@
       <c r="D11">
         <v>1</v>
       </c>
-      <c r="G11">
-        <f t="shared" ref="G11:G70" si="0">A11+2</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="12" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A12">
         <v>7</v>
       </c>
@@ -653,12 +645,8 @@
       <c r="D12">
         <v>1</v>
       </c>
-      <c r="G12">
-        <f t="shared" si="0"/>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="13" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A13">
         <v>8</v>
       </c>
@@ -671,12 +659,8 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="G13">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="14" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A14">
         <v>9</v>
       </c>
@@ -689,12 +673,8 @@
       <c r="D14">
         <v>1</v>
       </c>
-      <c r="G14">
-        <f t="shared" si="0"/>
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="15" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A15">
         <v>9</v>
       </c>
@@ -707,12 +687,8 @@
       <c r="D15">
         <v>1</v>
       </c>
-      <c r="G15">
-        <f t="shared" si="0"/>
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="16" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A16">
         <v>9</v>
       </c>
@@ -725,12 +701,8 @@
       <c r="D16">
         <v>1</v>
       </c>
-      <c r="G16">
-        <f t="shared" si="0"/>
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="17" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A17">
         <v>10</v>
       </c>
@@ -743,12 +715,8 @@
       <c r="D17">
         <v>1</v>
       </c>
-      <c r="G17">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="18" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A18">
         <v>10</v>
       </c>
@@ -761,12 +729,8 @@
       <c r="D18">
         <v>1</v>
       </c>
-      <c r="G18">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="19" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A19">
         <v>11</v>
       </c>
@@ -779,12 +743,8 @@
       <c r="D19">
         <v>1</v>
       </c>
-      <c r="G19">
-        <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="20" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A20">
         <v>11</v>
       </c>
@@ -797,12 +757,8 @@
       <c r="D20">
         <v>1</v>
       </c>
-      <c r="G20">
-        <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="21" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A21">
         <v>12</v>
       </c>
@@ -815,12 +771,8 @@
       <c r="D21">
         <v>1</v>
       </c>
-      <c r="G21">
-        <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="22" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A22">
         <v>12</v>
       </c>
@@ -833,12 +785,8 @@
       <c r="D22">
         <v>1</v>
       </c>
-      <c r="G22">
-        <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="23" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A23">
         <v>12</v>
       </c>
@@ -851,141 +799,109 @@
       <c r="D23">
         <v>1</v>
       </c>
-      <c r="G23">
-        <f t="shared" si="0"/>
+    </row>
+    <row r="24" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A24">
+        <v>13</v>
+      </c>
+      <c r="B24" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" t="s">
+        <v>7</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A25">
+        <v>13</v>
+      </c>
+      <c r="B25" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25" t="s">
+        <v>7</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A26">
         <v>14</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A24">
-        <v>14</v>
-      </c>
-      <c r="B24" t="s">
-        <v>6</v>
-      </c>
-      <c r="C24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D24">
-        <v>1</v>
-      </c>
-      <c r="G24">
-        <f t="shared" si="0"/>
+      <c r="B26" t="s">
+        <v>6</v>
+      </c>
+      <c r="C26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A27">
+        <v>15</v>
+      </c>
+      <c r="B27" t="s">
+        <v>8</v>
+      </c>
+      <c r="C27" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A28">
         <v>16</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A25">
-        <v>15</v>
-      </c>
-      <c r="B25" t="s">
-        <v>8</v>
-      </c>
-      <c r="C25" t="s">
-        <v>7</v>
-      </c>
-      <c r="D25">
-        <v>10</v>
-      </c>
-      <c r="G25">
-        <f t="shared" si="0"/>
-        <v>17</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A26">
-        <v>16</v>
-      </c>
-      <c r="B26" t="s">
-        <v>6</v>
-      </c>
-      <c r="C26" t="s">
-        <v>7</v>
-      </c>
-      <c r="D26">
-        <v>1</v>
-      </c>
-      <c r="G26">
-        <f t="shared" si="0"/>
+      <c r="B28" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A29">
         <v>18</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A27">
-        <v>17</v>
-      </c>
-      <c r="B27" t="s">
-        <v>9</v>
-      </c>
-      <c r="C27" t="s">
-        <v>14</v>
-      </c>
-      <c r="E27">
-        <v>-15</v>
-      </c>
-      <c r="G27">
-        <f t="shared" si="0"/>
+      <c r="B29" t="s">
+        <v>6</v>
+      </c>
+      <c r="C29" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A30">
         <v>19</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A28">
-        <v>18</v>
-      </c>
-      <c r="B28" t="s">
-        <v>6</v>
-      </c>
-      <c r="C28" t="s">
-        <v>7</v>
-      </c>
-      <c r="D28">
-        <v>1</v>
-      </c>
-      <c r="G28">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A29">
-        <v>19</v>
-      </c>
-      <c r="B29" t="s">
+      <c r="B30" t="s">
         <v>11</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C30" t="s">
         <v>12</v>
       </c>
-      <c r="D29">
+      <c r="D30">
         <v>30</v>
       </c>
-      <c r="F29">
-        <v>1</v>
-      </c>
-      <c r="G29">
-        <f t="shared" si="0"/>
-        <v>21</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A30">
-        <v>20</v>
-      </c>
-      <c r="B30" t="s">
-        <v>6</v>
-      </c>
-      <c r="C30" t="s">
-        <v>7</v>
-      </c>
-      <c r="D30">
-        <v>1</v>
-      </c>
-      <c r="G30">
-        <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="F30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A31">
         <v>20</v>
       </c>
@@ -998,231 +914,179 @@
       <c r="D31">
         <v>1</v>
       </c>
-      <c r="G31">
-        <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="32" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A32">
+        <v>20</v>
+      </c>
+      <c r="B32" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32" t="s">
+        <v>7</v>
+      </c>
+      <c r="D32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A33">
+        <v>20</v>
+      </c>
+      <c r="B33" t="s">
+        <v>6</v>
+      </c>
+      <c r="C33" t="s">
+        <v>7</v>
+      </c>
+      <c r="D33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A34">
+        <v>20</v>
+      </c>
+      <c r="B34" t="s">
+        <v>6</v>
+      </c>
+      <c r="C34" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A35">
         <v>21</v>
       </c>
-      <c r="B32" t="s">
-        <v>6</v>
-      </c>
-      <c r="C32" t="s">
-        <v>7</v>
-      </c>
-      <c r="D32">
-        <v>1</v>
-      </c>
-      <c r="G32">
-        <f t="shared" si="0"/>
+      <c r="B35" t="s">
+        <v>6</v>
+      </c>
+      <c r="C35" t="s">
+        <v>7</v>
+      </c>
+      <c r="D35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A36">
+        <v>21</v>
+      </c>
+      <c r="B36" t="s">
+        <v>6</v>
+      </c>
+      <c r="C36" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A37">
         <v>23</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A33">
-        <v>21</v>
-      </c>
-      <c r="B33" t="s">
-        <v>6</v>
-      </c>
-      <c r="C33" t="s">
-        <v>7</v>
-      </c>
-      <c r="D33">
-        <v>1</v>
-      </c>
-      <c r="G33">
-        <f t="shared" si="0"/>
-        <v>23</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A34">
-        <v>22</v>
-      </c>
-      <c r="B34" t="s">
-        <v>6</v>
-      </c>
-      <c r="C34" t="s">
-        <v>7</v>
-      </c>
-      <c r="D34">
-        <v>1</v>
-      </c>
-      <c r="G34">
-        <f t="shared" si="0"/>
-        <v>24</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A35">
-        <v>22</v>
-      </c>
-      <c r="B35" t="s">
-        <v>6</v>
-      </c>
-      <c r="C35" t="s">
-        <v>7</v>
-      </c>
-      <c r="D35">
-        <v>1</v>
-      </c>
-      <c r="G35">
-        <f t="shared" si="0"/>
-        <v>24</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A36">
-        <v>22</v>
-      </c>
-      <c r="B36" t="s">
-        <v>6</v>
-      </c>
-      <c r="C36" t="s">
-        <v>7</v>
-      </c>
-      <c r="D36">
-        <v>1</v>
-      </c>
-      <c r="G36">
-        <f t="shared" si="0"/>
-        <v>24</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A37">
-        <v>22</v>
-      </c>
       <c r="B37" t="s">
+        <v>9</v>
+      </c>
+      <c r="C37" t="s">
+        <v>14</v>
+      </c>
+      <c r="E37">
+        <v>-120</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A38">
+        <v>25</v>
+      </c>
+      <c r="B38" t="s">
+        <v>6</v>
+      </c>
+      <c r="C38" t="s">
+        <v>7</v>
+      </c>
+      <c r="D38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A39">
+        <v>25</v>
+      </c>
+      <c r="B39" t="s">
+        <v>6</v>
+      </c>
+      <c r="C39" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A40">
+        <v>25</v>
+      </c>
+      <c r="B40" t="s">
+        <v>6</v>
+      </c>
+      <c r="C40" t="s">
+        <v>7</v>
+      </c>
+      <c r="D40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A41">
+        <v>25</v>
+      </c>
+      <c r="B41" t="s">
         <v>8</v>
       </c>
-      <c r="C37" t="s">
-        <v>7</v>
-      </c>
-      <c r="D37">
-        <v>10</v>
-      </c>
-      <c r="G37">
-        <f t="shared" si="0"/>
-        <v>24</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A38">
-        <v>22</v>
-      </c>
-      <c r="B38" t="s">
-        <v>6</v>
-      </c>
-      <c r="C38" t="s">
-        <v>7</v>
-      </c>
-      <c r="D38">
-        <v>1</v>
-      </c>
-      <c r="G38">
-        <f t="shared" si="0"/>
-        <v>24</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A39">
-        <v>24</v>
-      </c>
-      <c r="B39" t="s">
-        <v>6</v>
-      </c>
-      <c r="C39" t="s">
-        <v>7</v>
-      </c>
-      <c r="D39">
-        <v>1</v>
-      </c>
-      <c r="G39">
-        <f t="shared" si="0"/>
+      <c r="C41" t="s">
+        <v>7</v>
+      </c>
+      <c r="D41">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A42">
         <v>26</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A40">
-        <v>24</v>
-      </c>
-      <c r="B40" t="s">
-        <v>6</v>
-      </c>
-      <c r="C40" t="s">
-        <v>7</v>
-      </c>
-      <c r="D40">
-        <v>1</v>
-      </c>
-      <c r="G40">
-        <f t="shared" si="0"/>
+      <c r="B42" t="s">
+        <v>6</v>
+      </c>
+      <c r="C42" t="s">
+        <v>7</v>
+      </c>
+      <c r="D42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A43">
         <v>26</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A41">
-        <v>24</v>
-      </c>
-      <c r="B41" t="s">
-        <v>6</v>
-      </c>
-      <c r="C41" t="s">
-        <v>7</v>
-      </c>
-      <c r="D41">
-        <v>1</v>
-      </c>
-      <c r="G41">
-        <f t="shared" si="0"/>
+      <c r="B43" t="s">
+        <v>6</v>
+      </c>
+      <c r="C43" t="s">
+        <v>7</v>
+      </c>
+      <c r="D43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A44">
         <v>26</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A42">
-        <v>25</v>
-      </c>
-      <c r="B42" t="s">
-        <v>6</v>
-      </c>
-      <c r="C42" t="s">
-        <v>7</v>
-      </c>
-      <c r="D42">
-        <v>1</v>
-      </c>
-      <c r="G42">
-        <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A43">
-        <v>25</v>
-      </c>
-      <c r="B43" t="s">
-        <v>6</v>
-      </c>
-      <c r="C43" t="s">
-        <v>7</v>
-      </c>
-      <c r="D43">
-        <v>1</v>
-      </c>
-      <c r="G43">
-        <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A44">
-        <v>27</v>
-      </c>
       <c r="B44" t="s">
         <v>6</v>
       </c>
@@ -1232,14 +1096,10 @@
       <c r="D44">
         <v>1</v>
       </c>
-      <c r="G44">
-        <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="45" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A45">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B45" t="s">
         <v>6</v>
@@ -1250,14 +1110,10 @@
       <c r="D45">
         <v>1</v>
       </c>
-      <c r="G45">
-        <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="46" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A46">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B46" t="s">
         <v>6</v>
@@ -1268,32 +1124,24 @@
       <c r="D46">
         <v>1</v>
       </c>
-      <c r="G46">
-        <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="47" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A47">
         <v>27</v>
       </c>
       <c r="B47" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C47" t="s">
         <v>7</v>
       </c>
       <c r="D47">
-        <v>10</v>
-      </c>
-      <c r="G47">
-        <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A48">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B48" t="s">
         <v>6</v>
@@ -1304,12 +1152,8 @@
       <c r="D48">
         <v>1</v>
       </c>
-      <c r="G48">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="49" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A49">
         <v>28</v>
       </c>
@@ -1322,33 +1166,25 @@
       <c r="D49">
         <v>1</v>
       </c>
-      <c r="G49">
-        <f t="shared" si="0"/>
+    </row>
+    <row r="50" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A50">
+        <v>28</v>
+      </c>
+      <c r="B50" t="s">
+        <v>6</v>
+      </c>
+      <c r="C50" t="s">
+        <v>7</v>
+      </c>
+      <c r="D50">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A51">
         <v>30</v>
       </c>
-    </row>
-    <row r="50" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A50">
-        <v>29</v>
-      </c>
-      <c r="B50" t="s">
-        <v>6</v>
-      </c>
-      <c r="C50" t="s">
-        <v>7</v>
-      </c>
-      <c r="D50">
-        <v>1</v>
-      </c>
-      <c r="G50">
-        <f t="shared" si="0"/>
-        <v>31</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A51">
-        <v>29</v>
-      </c>
       <c r="B51" t="s">
         <v>6</v>
       </c>
@@ -1358,14 +1194,10 @@
       <c r="D51">
         <v>1</v>
       </c>
-      <c r="G51">
-        <f t="shared" si="0"/>
-        <v>31</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="52" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A52">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B52" t="s">
         <v>6</v>
@@ -1376,12 +1208,8 @@
       <c r="D52">
         <v>1</v>
       </c>
-      <c r="G52">
-        <f t="shared" si="0"/>
-        <v>31</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="53" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A53">
         <v>30</v>
       </c>
@@ -1394,53 +1222,38 @@
       <c r="D53">
         <v>1</v>
       </c>
-      <c r="G53">
-        <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="54" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A54">
         <v>30</v>
       </c>
       <c r="B54" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C54" t="s">
         <v>7</v>
       </c>
       <c r="D54">
-        <v>1</v>
-      </c>
-      <c r="G54">
-        <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A55">
         <v>31</v>
       </c>
       <c r="B55" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C55" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D55">
-        <v>120</v>
-      </c>
-      <c r="F55">
-        <v>2</v>
-      </c>
-      <c r="G55">
-        <f t="shared" si="0"/>
-        <v>33</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A56">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B56" t="s">
         <v>6</v>
@@ -1451,12 +1264,8 @@
       <c r="D56">
         <v>1</v>
       </c>
-      <c r="G56">
-        <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="57" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A57">
         <v>32</v>
       </c>
@@ -1469,69 +1278,53 @@
       <c r="D57">
         <v>1</v>
       </c>
-      <c r="G57">
-        <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="58" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A58">
+        <v>32</v>
+      </c>
+      <c r="B58" t="s">
+        <v>6</v>
+      </c>
+      <c r="C58" t="s">
+        <v>7</v>
+      </c>
+      <c r="D58">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A59">
+        <v>32</v>
+      </c>
+      <c r="B59" t="s">
+        <v>6</v>
+      </c>
+      <c r="C59" t="s">
+        <v>7</v>
+      </c>
+      <c r="D59">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A60">
         <v>33</v>
       </c>
-      <c r="B58" t="s">
-        <v>6</v>
-      </c>
-      <c r="C58" t="s">
-        <v>7</v>
-      </c>
-      <c r="D58">
-        <v>1</v>
-      </c>
-      <c r="G58">
-        <f t="shared" si="0"/>
-        <v>35</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A59">
+      <c r="B60" t="s">
+        <v>6</v>
+      </c>
+      <c r="C60" t="s">
+        <v>7</v>
+      </c>
+      <c r="D60">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A61">
         <v>33</v>
       </c>
-      <c r="B59" t="s">
-        <v>6</v>
-      </c>
-      <c r="C59" t="s">
-        <v>7</v>
-      </c>
-      <c r="D59">
-        <v>1</v>
-      </c>
-      <c r="G59">
-        <f t="shared" si="0"/>
-        <v>35</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A60">
-        <v>34</v>
-      </c>
-      <c r="B60" t="s">
-        <v>6</v>
-      </c>
-      <c r="C60" t="s">
-        <v>7</v>
-      </c>
-      <c r="D60">
-        <v>1</v>
-      </c>
-      <c r="G60">
-        <f t="shared" si="0"/>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
-      <c r="A61">
-        <v>34</v>
-      </c>
       <c r="B61" t="s">
         <v>6</v>
       </c>
@@ -1541,30 +1334,25 @@
       <c r="D61">
         <v>1</v>
       </c>
-      <c r="G61">
-        <f t="shared" si="0"/>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="62" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A62">
         <v>34</v>
       </c>
       <c r="B62" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C62" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D62">
-        <v>1</v>
-      </c>
-      <c r="G62">
-        <f t="shared" si="0"/>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+        <v>120</v>
+      </c>
+      <c r="F62">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A63">
         <v>35</v>
       </c>
@@ -1577,12 +1365,8 @@
       <c r="D63">
         <v>1</v>
       </c>
-      <c r="G63">
-        <f t="shared" si="0"/>
-        <v>37</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="64" spans="1:6" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A64">
         <v>35</v>
       </c>
@@ -1595,12 +1379,8 @@
       <c r="D64">
         <v>1</v>
       </c>
-      <c r="G64">
-        <f t="shared" si="0"/>
-        <v>37</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="65" spans="1:4" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A65">
         <v>36</v>
       </c>
@@ -1613,12 +1393,8 @@
       <c r="D65">
         <v>1</v>
       </c>
-      <c r="G65">
-        <f t="shared" si="0"/>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="66" spans="1:4" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A66">
         <v>36</v>
       </c>
@@ -1631,12 +1407,8 @@
       <c r="D66">
         <v>1</v>
       </c>
-      <c r="G66">
-        <f t="shared" si="0"/>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="67" spans="1:4" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A67">
         <v>37</v>
       </c>
@@ -1649,12 +1421,8 @@
       <c r="D67">
         <v>1</v>
       </c>
-      <c r="G67">
-        <f t="shared" si="0"/>
-        <v>39</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="68" spans="1:4" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A68">
         <v>37</v>
       </c>
@@ -1667,12 +1435,8 @@
       <c r="D68">
         <v>1</v>
       </c>
-      <c r="G68">
-        <f t="shared" si="0"/>
-        <v>39</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="69" spans="1:4" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A69">
         <v>37</v>
       </c>
@@ -1685,39 +1449,122 @@
       <c r="D69">
         <v>1</v>
       </c>
-      <c r="G69">
-        <f t="shared" si="0"/>
-        <v>39</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" ht="14.25" x14ac:dyDescent="0.15">
+    </row>
+    <row r="70" spans="1:4" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A70">
         <v>38</v>
       </c>
       <c r="B70" t="s">
+        <v>6</v>
+      </c>
+      <c r="C70" t="s">
+        <v>7</v>
+      </c>
+      <c r="D70">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A71">
+        <v>38</v>
+      </c>
+      <c r="B71" t="s">
+        <v>6</v>
+      </c>
+      <c r="C71" t="s">
+        <v>7</v>
+      </c>
+      <c r="D71">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A72">
+        <v>39</v>
+      </c>
+      <c r="B72" t="s">
+        <v>6</v>
+      </c>
+      <c r="C72" t="s">
+        <v>7</v>
+      </c>
+      <c r="D72">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A73">
+        <v>39</v>
+      </c>
+      <c r="B73" t="s">
+        <v>6</v>
+      </c>
+      <c r="C73" t="s">
+        <v>7</v>
+      </c>
+      <c r="D73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A74">
+        <v>40</v>
+      </c>
+      <c r="B74" t="s">
+        <v>6</v>
+      </c>
+      <c r="C74" t="s">
+        <v>7</v>
+      </c>
+      <c r="D74">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A75">
+        <v>40</v>
+      </c>
+      <c r="B75" t="s">
+        <v>6</v>
+      </c>
+      <c r="C75" t="s">
+        <v>7</v>
+      </c>
+      <c r="D75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A76">
+        <v>40</v>
+      </c>
+      <c r="B76" t="s">
+        <v>6</v>
+      </c>
+      <c r="C76" t="s">
+        <v>7</v>
+      </c>
+      <c r="D76">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" ht="14.25" x14ac:dyDescent="0.15">
+      <c r="A77">
+        <v>41</v>
+      </c>
+      <c r="B77" t="s">
         <v>13</v>
       </c>
-      <c r="C70" t="s">
+      <c r="C77" t="s">
         <v>12</v>
       </c>
-      <c r="D70">
+      <c r="D77">
         <v>1000</v>
       </c>
-      <c r="G70">
-        <f t="shared" si="0"/>
-        <v>40</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" ht="14.25" x14ac:dyDescent="0.15"/>
-    <row r="72" spans="1:7" ht="14.25" x14ac:dyDescent="0.15"/>
-    <row r="73" spans="1:7" ht="14.25" x14ac:dyDescent="0.15"/>
-    <row r="74" spans="1:7" ht="14.25" x14ac:dyDescent="0.15"/>
-    <row r="75" spans="1:7" ht="14.25" x14ac:dyDescent="0.15"/>
-    <row r="76" spans="1:7" ht="14.25" x14ac:dyDescent="0.15"/>
-    <row r="77" spans="1:7" ht="14.25" x14ac:dyDescent="0.15"/>
-    <row r="78" spans="1:7" ht="14.25" x14ac:dyDescent="0.15"/>
-    <row r="79" spans="1:7" ht="14.25" x14ac:dyDescent="0.15"/>
-    <row r="80" spans="1:7" ht="14.25" x14ac:dyDescent="0.15"/>
+    </row>
+    <row r="78" spans="1:4" ht="14.25" x14ac:dyDescent="0.15"/>
+    <row r="79" spans="1:4" ht="14.25" x14ac:dyDescent="0.15"/>
+    <row r="80" spans="1:4" ht="14.25" x14ac:dyDescent="0.15"/>
     <row r="81" ht="14.25" x14ac:dyDescent="0.15"/>
     <row r="82" ht="14.25" x14ac:dyDescent="0.15"/>
     <row r="83" ht="14.25" x14ac:dyDescent="0.15"/>
@@ -1730,12 +1577,19 @@
     <row r="90" ht="14.25" x14ac:dyDescent="0.15"/>
     <row r="91" ht="14.25" x14ac:dyDescent="0.15"/>
     <row r="92" ht="14.25" x14ac:dyDescent="0.15"/>
+    <row r="93" ht="14.25" x14ac:dyDescent="0.15"/>
+    <row r="94" ht="14.25" x14ac:dyDescent="0.15"/>
+    <row r="95" ht="14.25" x14ac:dyDescent="0.15"/>
+    <row r="96" ht="14.25" x14ac:dyDescent="0.15"/>
+    <row r="97" ht="14.25" x14ac:dyDescent="0.15"/>
+    <row r="98" ht="14.25" x14ac:dyDescent="0.15"/>
+    <row r="99" ht="14.25" x14ac:dyDescent="0.15"/>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="B10:F12 A1:F8 B14:F23 B13:F13 B29:F37 B39:F43 B44:F54 B56:F69 B27 B25:F25 B70:C70 E70:F70 D27:F27" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:F8 B10:F23 B38:F40 B47:F53 B63:F76 B27:C27 B77:C77 E77:F77 B35:F36 B30:F32 B43:F43 B41:C41 E41:F41 E27:F27 B55:F61 B54:C54 E54:F54" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: Final map sync, boss conditionals, UI polish
</commit_message>
<xml_diff>
--- a/av01/spawn_config.xlsx
+++ b/av01/spawn_config.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="15150" windowHeight="12735"/>
+    <workbookView windowWidth="15150" windowHeight="13455"/>
   </bookViews>
   <sheets>
     <sheet name="Spawns" sheetId="1" r:id="rId1"/>
@@ -87,14 +87,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="20">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -550,148 +543,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1154,7 +1147,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
@@ -1168,7 +1161,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
@@ -1182,7 +1175,7 @@
     </row>
     <row r="7" ht="17" customHeight="1" spans="1:4">
       <c r="A7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
         <v>6</v>
@@ -1196,7 +1189,7 @@
     </row>
     <row r="8" ht="15" customHeight="1" spans="1:4">
       <c r="A8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B8" t="s">
         <v>6</v>
@@ -1210,7 +1203,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B9" t="s">
         <v>6</v>
@@ -1224,7 +1217,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B10" t="s">
         <v>6</v>
@@ -1238,7 +1231,7 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B11" t="s">
         <v>6</v>
@@ -1252,7 +1245,7 @@
     </row>
     <row r="12" customFormat="1" spans="1:4">
       <c r="A12">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B12" t="s">
         <v>11</v>
@@ -1266,7 +1259,7 @@
     </row>
     <row r="13" customFormat="1" spans="1:4">
       <c r="A13">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B13" t="s">
         <v>11</v>
@@ -1280,7 +1273,7 @@
     </row>
     <row r="14" customFormat="1" spans="1:6">
       <c r="A14">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B14" t="s">
         <v>12</v>
@@ -1297,7 +1290,7 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B15" t="s">
         <v>6</v>
@@ -1311,7 +1304,7 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B16" t="s">
         <v>6</v>
@@ -1325,7 +1318,7 @@
     </row>
     <row r="17" spans="1:4">
       <c r="A17">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B17" t="s">
         <v>6</v>
@@ -1339,7 +1332,7 @@
     </row>
     <row r="18" customFormat="1" spans="1:4">
       <c r="A18">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B18" t="s">
         <v>11</v>
@@ -1353,7 +1346,7 @@
     </row>
     <row r="19" customFormat="1" spans="1:4">
       <c r="A19">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B19" t="s">
         <v>11</v>
@@ -1367,7 +1360,7 @@
     </row>
     <row r="20" customFormat="1" spans="1:4">
       <c r="A20">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B20" t="s">
         <v>11</v>
@@ -1381,7 +1374,7 @@
     </row>
     <row r="21" customFormat="1" spans="1:4">
       <c r="A21">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B21" t="s">
         <v>11</v>
@@ -1395,7 +1388,7 @@
     </row>
     <row r="22" customFormat="1" spans="1:4">
       <c r="A22">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B22" t="s">
         <v>11</v>
@@ -1409,7 +1402,7 @@
     </row>
     <row r="23" customFormat="1" spans="1:4">
       <c r="A23">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B23" t="s">
         <v>11</v>
@@ -1423,7 +1416,7 @@
     </row>
     <row r="24" customFormat="1" spans="1:4">
       <c r="A24">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B24" t="s">
         <v>6</v>
@@ -1437,7 +1430,7 @@
     </row>
     <row r="25" customFormat="1" spans="1:4">
       <c r="A25">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B25" t="s">
         <v>6</v>
@@ -1451,7 +1444,7 @@
     </row>
     <row r="26" customFormat="1" spans="1:4">
       <c r="A26">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B26" t="s">
         <v>6</v>
@@ -1465,7 +1458,7 @@
     </row>
     <row r="27" customFormat="1" spans="1:4">
       <c r="A27">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B27" t="s">
         <v>6</v>
@@ -1479,7 +1472,7 @@
     </row>
     <row r="28" customFormat="1" spans="1:4">
       <c r="A28">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B28" t="s">
         <v>6</v>
@@ -1493,7 +1486,7 @@
     </row>
     <row r="29" customFormat="1" spans="1:4">
       <c r="A29">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B29" t="s">
         <v>6</v>
@@ -1507,7 +1500,7 @@
     </row>
     <row r="30" customFormat="1" spans="1:4">
       <c r="A30">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B30" t="s">
         <v>6</v>
@@ -1521,7 +1514,7 @@
     </row>
     <row r="31" customFormat="1" spans="1:4">
       <c r="A31">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B31" t="s">
         <v>11</v>
@@ -1535,7 +1528,7 @@
     </row>
     <row r="32" customFormat="1" spans="1:4">
       <c r="A32">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B32" t="s">
         <v>11</v>
@@ -1549,7 +1542,7 @@
     </row>
     <row r="33" customFormat="1" spans="1:4">
       <c r="A33">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B33" t="s">
         <v>11</v>
@@ -1563,7 +1556,7 @@
     </row>
     <row r="34" customFormat="1" spans="1:4">
       <c r="A34">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B34" t="s">
         <v>11</v>
@@ -1577,7 +1570,7 @@
     </row>
     <row r="35" customFormat="1" spans="1:4">
       <c r="A35">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B35" t="s">
         <v>11</v>
@@ -1591,7 +1584,7 @@
     </row>
     <row r="36" customFormat="1" spans="1:4">
       <c r="A36">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B36" t="s">
         <v>11</v>
@@ -1605,7 +1598,7 @@
     </row>
     <row r="37" customFormat="1" spans="1:4">
       <c r="A37">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B37" t="s">
         <v>11</v>
@@ -1619,7 +1612,7 @@
     </row>
     <row r="38" customFormat="1" spans="1:4">
       <c r="A38">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B38" t="s">
         <v>6</v>
@@ -1633,7 +1626,7 @@
     </row>
     <row r="39" customFormat="1" spans="1:4">
       <c r="A39">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B39" t="s">
         <v>6</v>
@@ -1647,7 +1640,7 @@
     </row>
     <row r="40" customFormat="1" spans="1:4">
       <c r="A40">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B40" t="s">
         <v>6</v>
@@ -1661,7 +1654,7 @@
     </row>
     <row r="41" customFormat="1" spans="1:4">
       <c r="A41">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B41" t="s">
         <v>6</v>
@@ -1675,7 +1668,7 @@
     </row>
     <row r="42" customFormat="1" spans="1:4">
       <c r="A42">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B42" t="s">
         <v>6</v>
@@ -1689,7 +1682,7 @@
     </row>
     <row r="43" customFormat="1" spans="1:4">
       <c r="A43">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B43" t="s">
         <v>6</v>
@@ -1703,7 +1696,7 @@
     </row>
     <row r="44" customFormat="1" spans="1:4">
       <c r="A44">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B44" t="s">
         <v>6</v>
@@ -1717,7 +1710,7 @@
     </row>
     <row r="45" customFormat="1" spans="1:4">
       <c r="A45">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B45" t="s">
         <v>6</v>
@@ -1731,7 +1724,7 @@
     </row>
     <row r="46" customFormat="1" spans="1:4">
       <c r="A46">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B46" t="s">
         <v>6</v>
@@ -1745,7 +1738,7 @@
     </row>
     <row r="47" customFormat="1" spans="1:4">
       <c r="A47">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B47" t="s">
         <v>6</v>
@@ -1759,7 +1752,7 @@
     </row>
     <row r="48" customFormat="1" spans="1:4">
       <c r="A48">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B48" t="s">
         <v>6</v>
@@ -1773,7 +1766,7 @@
     </row>
     <row r="49" customFormat="1" spans="1:4">
       <c r="A49">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B49" t="s">
         <v>6</v>
@@ -1787,7 +1780,7 @@
     </row>
     <row r="50" customFormat="1" spans="1:4">
       <c r="A50">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B50" t="s">
         <v>11</v>
@@ -1801,7 +1794,7 @@
     </row>
     <row r="51" customFormat="1" spans="1:4">
       <c r="A51">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B51" t="s">
         <v>11</v>
@@ -1815,7 +1808,7 @@
     </row>
     <row r="52" customFormat="1" spans="1:4">
       <c r="A52">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B52" t="s">
         <v>11</v>
@@ -1829,7 +1822,7 @@
     </row>
     <row r="53" customFormat="1" spans="1:4">
       <c r="A53">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B53" t="s">
         <v>11</v>
@@ -1843,7 +1836,7 @@
     </row>
     <row r="54" customFormat="1" spans="1:4">
       <c r="A54">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B54" t="s">
         <v>6</v>
@@ -1857,7 +1850,7 @@
     </row>
     <row r="55" customFormat="1" spans="1:4">
       <c r="A55">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B55" t="s">
         <v>6</v>
@@ -1871,7 +1864,7 @@
     </row>
     <row r="56" customFormat="1" spans="1:4">
       <c r="A56">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B56" t="s">
         <v>6</v>
@@ -1885,7 +1878,7 @@
     </row>
     <row r="57" customFormat="1" spans="1:4">
       <c r="A57">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B57" t="s">
         <v>6</v>
@@ -1899,7 +1892,7 @@
     </row>
     <row r="58" customFormat="1" spans="1:4">
       <c r="A58">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B58" t="s">
         <v>6</v>
@@ -1913,7 +1906,7 @@
     </row>
     <row r="59" customFormat="1" spans="1:4">
       <c r="A59">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B59" t="s">
         <v>14</v>
@@ -1927,7 +1920,7 @@
     </row>
     <row r="60" customFormat="1" spans="1:4">
       <c r="A60">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B60" t="s">
         <v>6</v>
@@ -1941,7 +1934,7 @@
     </row>
     <row r="61" customFormat="1" spans="1:6">
       <c r="A61">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B61" t="s">
         <v>12</v>
@@ -1958,7 +1951,7 @@
     </row>
     <row r="62" customFormat="1" spans="1:4">
       <c r="A62">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B62" t="s">
         <v>14</v>
@@ -1972,7 +1965,7 @@
     </row>
     <row r="63" spans="1:4">
       <c r="A63">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B63" t="s">
         <v>6</v>
@@ -1986,7 +1979,7 @@
     </row>
     <row r="64" spans="1:4">
       <c r="A64">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B64" t="s">
         <v>6</v>
@@ -2000,7 +1993,7 @@
     </row>
     <row r="65" customFormat="1" spans="1:4">
       <c r="A65">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B65" t="s">
         <v>6</v>
@@ -2014,7 +2007,7 @@
     </row>
     <row r="66" customFormat="1" spans="1:4">
       <c r="A66">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B66" t="s">
         <v>6</v>
@@ -2028,7 +2021,7 @@
     </row>
     <row r="67" customFormat="1" ht="16" customHeight="1" spans="1:4">
       <c r="A67">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B67" t="s">
         <v>6</v>
@@ -2042,7 +2035,7 @@
     </row>
     <row r="68" customFormat="1" spans="1:4">
       <c r="A68">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B68" t="s">
         <v>14</v>
@@ -2056,7 +2049,7 @@
     </row>
     <row r="69" customFormat="1" spans="1:4">
       <c r="A69">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B69" t="s">
         <v>6</v>
@@ -2070,7 +2063,7 @@
     </row>
     <row r="70" customFormat="1" spans="1:4">
       <c r="A70">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B70" t="s">
         <v>6</v>
@@ -2084,7 +2077,7 @@
     </row>
     <row r="71" customFormat="1" spans="1:4">
       <c r="A71">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B71" t="s">
         <v>14</v>
@@ -2098,7 +2091,7 @@
     </row>
     <row r="72" customFormat="1" spans="1:4">
       <c r="A72">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B72" t="s">
         <v>6</v>
@@ -2112,7 +2105,7 @@
     </row>
     <row r="73" customFormat="1" ht="16" customHeight="1" spans="1:4">
       <c r="A73">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B73" t="s">
         <v>14</v>
@@ -2126,7 +2119,7 @@
     </row>
     <row r="74" customFormat="1" spans="1:4">
       <c r="A74">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B74" t="s">
         <v>6</v>
@@ -2140,7 +2133,7 @@
     </row>
     <row r="75" customFormat="1" spans="1:4">
       <c r="A75">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B75" t="s">
         <v>6</v>
@@ -2154,7 +2147,7 @@
     </row>
     <row r="76" customFormat="1" spans="1:4">
       <c r="A76">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B76" t="s">
         <v>6</v>
@@ -2168,7 +2161,7 @@
     </row>
     <row r="77" customFormat="1" spans="1:4">
       <c r="A77">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B77" t="s">
         <v>14</v>
@@ -2182,7 +2175,7 @@
     </row>
     <row r="78" customFormat="1" spans="1:4">
       <c r="A78">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B78" t="s">
         <v>6</v>
@@ -2196,7 +2189,7 @@
     </row>
     <row r="79" customFormat="1" spans="1:4">
       <c r="A79">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B79" t="s">
         <v>6</v>
@@ -2210,7 +2203,7 @@
     </row>
     <row r="80" customFormat="1" spans="1:4">
       <c r="A80">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B80" t="s">
         <v>6</v>
@@ -2224,7 +2217,7 @@
     </row>
     <row r="81" customFormat="1" spans="1:4">
       <c r="A81">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B81" t="s">
         <v>14</v>
@@ -2238,7 +2231,7 @@
     </row>
     <row r="82" customFormat="1" spans="1:4">
       <c r="A82">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B82" t="s">
         <v>6</v>
@@ -2252,7 +2245,7 @@
     </row>
     <row r="83" customFormat="1" spans="1:5">
       <c r="A83">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B83" t="s">
         <v>8</v>
@@ -2267,7 +2260,7 @@
     </row>
     <row r="84" customFormat="1" spans="1:4">
       <c r="A84">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B84" t="s">
         <v>11</v>
@@ -2281,7 +2274,7 @@
     </row>
     <row r="85" customFormat="1" spans="1:4">
       <c r="A85">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B85" t="s">
         <v>11</v>
@@ -2295,7 +2288,7 @@
     </row>
     <row r="86" customFormat="1" spans="1:4">
       <c r="A86">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B86" t="s">
         <v>11</v>
@@ -2309,7 +2302,7 @@
     </row>
     <row r="87" customFormat="1" spans="1:4">
       <c r="A87">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B87" t="s">
         <v>11</v>
@@ -2323,7 +2316,7 @@
     </row>
     <row r="88" customFormat="1" spans="1:4">
       <c r="A88">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B88" t="s">
         <v>11</v>
@@ -2337,7 +2330,7 @@
     </row>
     <row r="89" customFormat="1" spans="1:4">
       <c r="A89">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B89" t="s">
         <v>11</v>
@@ -2351,7 +2344,7 @@
     </row>
     <row r="90" customFormat="1" spans="1:4">
       <c r="A90">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B90" t="s">
         <v>11</v>
@@ -2365,7 +2358,7 @@
     </row>
     <row r="91" customFormat="1" spans="1:4">
       <c r="A91">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B91" t="s">
         <v>11</v>
@@ -2379,7 +2372,7 @@
     </row>
     <row r="92" customFormat="1" spans="1:4">
       <c r="A92">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B92" t="s">
         <v>14</v>
@@ -2393,7 +2386,7 @@
     </row>
     <row r="93" customFormat="1" spans="1:4">
       <c r="A93">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B93" t="s">
         <v>14</v>
@@ -2407,7 +2400,7 @@
     </row>
     <row r="94" customFormat="1" spans="1:4">
       <c r="A94">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B94" t="s">
         <v>14</v>
@@ -2421,7 +2414,7 @@
     </row>
     <row r="95" customFormat="1" spans="1:4">
       <c r="A95">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B95" t="s">
         <v>14</v>
@@ -2435,7 +2428,7 @@
     </row>
     <row r="96" customFormat="1" spans="1:4">
       <c r="A96">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B96" t="s">
         <v>14</v>
@@ -2449,7 +2442,7 @@
     </row>
     <row r="97" customFormat="1" spans="1:4">
       <c r="A97">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B97" t="s">
         <v>14</v>
@@ -2463,7 +2456,7 @@
     </row>
     <row r="98" customFormat="1" spans="1:4">
       <c r="A98">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B98" t="s">
         <v>14</v>
@@ -2477,7 +2470,7 @@
     </row>
     <row r="99" customFormat="1" spans="1:4">
       <c r="A99">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B99" t="s">
         <v>11</v>
@@ -2491,7 +2484,7 @@
     </row>
     <row r="100" customFormat="1" spans="1:4">
       <c r="A100">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B100" t="s">
         <v>11</v>
@@ -2505,7 +2498,7 @@
     </row>
     <row r="101" customFormat="1" spans="1:4">
       <c r="A101">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B101" t="s">
         <v>11</v>
@@ -2519,7 +2512,7 @@
     </row>
     <row r="102" customFormat="1" spans="1:4">
       <c r="A102">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B102" t="s">
         <v>11</v>
@@ -2533,7 +2526,7 @@
     </row>
     <row r="103" customFormat="1" spans="1:4">
       <c r="A103">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B103" t="s">
         <v>11</v>
@@ -2547,7 +2540,7 @@
     </row>
     <row r="104" customFormat="1" spans="1:4">
       <c r="A104">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B104" t="s">
         <v>11</v>
@@ -2561,7 +2554,7 @@
     </row>
     <row r="105" customFormat="1" spans="1:4">
       <c r="A105">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B105" t="s">
         <v>11</v>
@@ -2575,7 +2568,7 @@
     </row>
     <row r="106" customFormat="1" spans="1:4">
       <c r="A106">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B106" t="s">
         <v>11</v>
@@ -2589,7 +2582,7 @@
     </row>
     <row r="107" customFormat="1" spans="1:4">
       <c r="A107">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B107" t="s">
         <v>14</v>
@@ -2603,7 +2596,7 @@
     </row>
     <row r="108" customFormat="1" spans="1:4">
       <c r="A108">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B108" t="s">
         <v>14</v>
@@ -2617,7 +2610,7 @@
     </row>
     <row r="109" customFormat="1" spans="1:4">
       <c r="A109">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B109" t="s">
         <v>14</v>
@@ -2631,7 +2624,7 @@
     </row>
     <row r="110" customFormat="1" spans="1:4">
       <c r="A110">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B110" t="s">
         <v>14</v>
@@ -2645,7 +2638,7 @@
     </row>
     <row r="111" customFormat="1" spans="1:4">
       <c r="A111">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B111" t="s">
         <v>14</v>
@@ -2659,7 +2652,7 @@
     </row>
     <row r="112" customFormat="1" spans="1:4">
       <c r="A112">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B112" t="s">
         <v>14</v>
@@ -2673,7 +2666,7 @@
     </row>
     <row r="113" customFormat="1" spans="1:4">
       <c r="A113">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B113" t="s">
         <v>14</v>
@@ -2687,7 +2680,7 @@
     </row>
     <row r="114" customFormat="1" spans="1:4">
       <c r="A114">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B114" t="s">
         <v>14</v>
@@ -2701,7 +2694,7 @@
     </row>
     <row r="115" customFormat="1" spans="1:4">
       <c r="A115">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B115" t="s">
         <v>14</v>
@@ -2715,7 +2708,7 @@
     </row>
     <row r="116" customFormat="1" spans="1:4">
       <c r="A116">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B116" t="s">
         <v>11</v>
@@ -2729,7 +2722,7 @@
     </row>
     <row r="117" customFormat="1" spans="1:4">
       <c r="A117">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B117" t="s">
         <v>11</v>
@@ -2743,7 +2736,7 @@
     </row>
     <row r="118" customFormat="1" spans="1:4">
       <c r="A118">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B118" t="s">
         <v>11</v>
@@ -2757,7 +2750,7 @@
     </row>
     <row r="119" customFormat="1" spans="1:4">
       <c r="A119">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B119" t="s">
         <v>11</v>
@@ -2771,7 +2764,7 @@
     </row>
     <row r="120" customFormat="1" spans="1:4">
       <c r="A120">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B120" t="s">
         <v>11</v>
@@ -2785,7 +2778,7 @@
     </row>
     <row r="121" customFormat="1" spans="1:4">
       <c r="A121">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B121" t="s">
         <v>11</v>
@@ -2799,7 +2792,7 @@
     </row>
     <row r="122" customFormat="1" spans="1:4">
       <c r="A122">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B122" t="s">
         <v>11</v>
@@ -2813,7 +2806,7 @@
     </row>
     <row r="123" customFormat="1" spans="1:4">
       <c r="A123">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B123" t="s">
         <v>11</v>
@@ -2827,7 +2820,7 @@
     </row>
     <row r="124" customFormat="1" spans="1:4">
       <c r="A124">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B124" t="s">
         <v>14</v>
@@ -2841,7 +2834,7 @@
     </row>
     <row r="125" customFormat="1" spans="1:4">
       <c r="A125">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B125" t="s">
         <v>6</v>
@@ -2855,7 +2848,7 @@
     </row>
     <row r="126" customFormat="1" spans="1:4">
       <c r="A126">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B126" t="s">
         <v>14</v>
@@ -2869,7 +2862,7 @@
     </row>
     <row r="127" customFormat="1" spans="1:4">
       <c r="A127">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B127" t="s">
         <v>6</v>
@@ -2883,7 +2876,7 @@
     </row>
     <row r="128" customFormat="1" spans="1:4">
       <c r="A128">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B128" t="s">
         <v>14</v>
@@ -2897,7 +2890,7 @@
     </row>
     <row r="129" customFormat="1" spans="1:4">
       <c r="A129">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B129" t="s">
         <v>6</v>
@@ -2911,7 +2904,7 @@
     </row>
     <row r="130" customFormat="1" spans="1:4">
       <c r="A130">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B130" t="s">
         <v>14</v>
@@ -2925,7 +2918,7 @@
     </row>
     <row r="131" customFormat="1" spans="1:4">
       <c r="A131">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B131" t="s">
         <v>11</v>
@@ -2939,7 +2932,7 @@
     </row>
     <row r="132" customFormat="1" spans="1:4">
       <c r="A132">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B132" t="s">
         <v>11</v>
@@ -2953,7 +2946,7 @@
     </row>
     <row r="133" customFormat="1" spans="1:4">
       <c r="A133">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B133" t="s">
         <v>11</v>
@@ -2967,7 +2960,7 @@
     </row>
     <row r="134" customFormat="1" spans="1:4">
       <c r="A134">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B134" t="s">
         <v>11</v>
@@ -2981,7 +2974,7 @@
     </row>
     <row r="135" customFormat="1" spans="1:4">
       <c r="A135">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B135" t="s">
         <v>11</v>
@@ -2995,7 +2988,7 @@
     </row>
     <row r="136" customFormat="1" spans="1:4">
       <c r="A136">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B136" t="s">
         <v>11</v>
@@ -3009,7 +3002,7 @@
     </row>
     <row r="137" customFormat="1" spans="1:4">
       <c r="A137">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B137" t="s">
         <v>11</v>
@@ -3023,7 +3016,7 @@
     </row>
     <row r="138" customFormat="1" spans="1:4">
       <c r="A138">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B138" t="s">
         <v>11</v>
@@ -3037,7 +3030,7 @@
     </row>
     <row r="139" customFormat="1" spans="1:4">
       <c r="A139">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B139" t="s">
         <v>14</v>
@@ -3051,7 +3044,7 @@
     </row>
     <row r="140" customFormat="1" spans="1:4">
       <c r="A140">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B140" t="s">
         <v>6</v>
@@ -3065,7 +3058,7 @@
     </row>
     <row r="141" customFormat="1" spans="1:4">
       <c r="A141">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B141" t="s">
         <v>14</v>
@@ -3079,7 +3072,7 @@
     </row>
     <row r="142" customFormat="1" spans="1:4">
       <c r="A142">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B142" t="s">
         <v>6</v>
@@ -3093,7 +3086,7 @@
     </row>
     <row r="143" customFormat="1" spans="1:4">
       <c r="A143">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B143" t="s">
         <v>14</v>
@@ -3107,7 +3100,7 @@
     </row>
     <row r="144" customFormat="1" spans="1:4">
       <c r="A144">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B144" t="s">
         <v>6</v>
@@ -3121,7 +3114,7 @@
     </row>
     <row r="145" customFormat="1" spans="1:4">
       <c r="A145">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B145" t="s">
         <v>14</v>
@@ -3135,7 +3128,7 @@
     </row>
     <row r="146" customFormat="1" spans="1:4">
       <c r="A146">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B146" t="s">
         <v>11</v>
@@ -3149,7 +3142,7 @@
     </row>
     <row r="147" customFormat="1" spans="1:4">
       <c r="A147">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B147" t="s">
         <v>11</v>
@@ -3163,7 +3156,7 @@
     </row>
     <row r="148" customFormat="1" spans="1:4">
       <c r="A148">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B148" t="s">
         <v>11</v>
@@ -3177,7 +3170,7 @@
     </row>
     <row r="149" customFormat="1" spans="1:4">
       <c r="A149">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B149" t="s">
         <v>11</v>
@@ -3191,7 +3184,7 @@
     </row>
     <row r="150" customFormat="1" spans="1:4">
       <c r="A150">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B150" t="s">
         <v>11</v>
@@ -3205,7 +3198,7 @@
     </row>
     <row r="151" customFormat="1" spans="1:4">
       <c r="A151">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B151" t="s">
         <v>11</v>
@@ -3219,7 +3212,7 @@
     </row>
     <row r="152" customFormat="1" spans="1:4">
       <c r="A152">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B152" t="s">
         <v>11</v>
@@ -3233,7 +3226,7 @@
     </row>
     <row r="153" customFormat="1" spans="1:4">
       <c r="A153">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B153" t="s">
         <v>11</v>
@@ -3247,7 +3240,7 @@
     </row>
     <row r="154" customFormat="1" spans="1:4">
       <c r="A154">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B154" t="s">
         <v>14</v>
@@ -3261,7 +3254,7 @@
     </row>
     <row r="155" customFormat="1" spans="1:4">
       <c r="A155">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B155" t="s">
         <v>6</v>
@@ -3275,7 +3268,7 @@
     </row>
     <row r="156" customFormat="1" spans="1:4">
       <c r="A156">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B156" t="s">
         <v>14</v>
@@ -3289,7 +3282,7 @@
     </row>
     <row r="157" customFormat="1" spans="1:4">
       <c r="A157">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B157" t="s">
         <v>6</v>
@@ -3303,7 +3296,7 @@
     </row>
     <row r="158" customFormat="1" spans="1:4">
       <c r="A158">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B158" t="s">
         <v>14</v>
@@ -3317,7 +3310,7 @@
     </row>
     <row r="159" customFormat="1" spans="1:4">
       <c r="A159">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B159" t="s">
         <v>6</v>
@@ -3331,7 +3324,7 @@
     </row>
     <row r="160" customFormat="1" spans="1:4">
       <c r="A160">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B160" t="s">
         <v>14</v>
@@ -3345,7 +3338,7 @@
     </row>
     <row r="161" customFormat="1" spans="1:4">
       <c r="A161">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B161" t="s">
         <v>11</v>
@@ -3359,7 +3352,7 @@
     </row>
     <row r="162" customFormat="1" spans="1:4">
       <c r="A162">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B162" t="s">
         <v>11</v>
@@ -3373,7 +3366,7 @@
     </row>
     <row r="163" customFormat="1" spans="1:4">
       <c r="A163">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B163" t="s">
         <v>11</v>
@@ -3387,7 +3380,7 @@
     </row>
     <row r="164" customFormat="1" spans="1:4">
       <c r="A164">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B164" t="s">
         <v>11</v>
@@ -3401,7 +3394,7 @@
     </row>
     <row r="165" customFormat="1" spans="1:4">
       <c r="A165">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B165" t="s">
         <v>11</v>
@@ -3415,7 +3408,7 @@
     </row>
     <row r="166" customFormat="1" spans="1:4">
       <c r="A166">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B166" t="s">
         <v>11</v>
@@ -3429,7 +3422,7 @@
     </row>
     <row r="167" customFormat="1" spans="1:4">
       <c r="A167">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B167" t="s">
         <v>11</v>
@@ -3443,7 +3436,7 @@
     </row>
     <row r="168" customFormat="1" spans="1:4">
       <c r="A168">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B168" t="s">
         <v>11</v>
@@ -3457,7 +3450,7 @@
     </row>
     <row r="169" customFormat="1" spans="1:4">
       <c r="A169">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B169" t="s">
         <v>14</v>
@@ -3471,7 +3464,7 @@
     </row>
     <row r="170" customFormat="1" spans="1:4">
       <c r="A170">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B170" t="s">
         <v>6</v>
@@ -3485,7 +3478,7 @@
     </row>
     <row r="171" customFormat="1" spans="1:4">
       <c r="A171">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B171" t="s">
         <v>14</v>
@@ -3499,7 +3492,7 @@
     </row>
     <row r="172" customFormat="1" spans="1:4">
       <c r="A172">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B172" t="s">
         <v>6</v>
@@ -3513,7 +3506,7 @@
     </row>
     <row r="173" customFormat="1" spans="1:4">
       <c r="A173">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B173" t="s">
         <v>14</v>
@@ -3527,7 +3520,7 @@
     </row>
     <row r="174" customFormat="1" spans="1:4">
       <c r="A174">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B174" t="s">
         <v>6</v>
@@ -3541,7 +3534,7 @@
     </row>
     <row r="175" customFormat="1" ht="15" customHeight="1" spans="1:4">
       <c r="A175">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B175" t="s">
         <v>14</v>
@@ -3555,7 +3548,7 @@
     </row>
     <row r="176" customFormat="1" spans="1:4">
       <c r="A176">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B176" t="s">
         <v>14</v>
@@ -3569,7 +3562,7 @@
     </row>
     <row r="177" customFormat="1" spans="1:4">
       <c r="A177">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B177" t="s">
         <v>6</v>
@@ -3583,7 +3576,7 @@
     </row>
     <row r="178" customFormat="1" spans="1:4">
       <c r="A178">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B178" t="s">
         <v>14</v>
@@ -3597,7 +3590,7 @@
     </row>
     <row r="179" customFormat="1" spans="1:4">
       <c r="A179">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B179" t="s">
         <v>6</v>
@@ -3611,7 +3604,7 @@
     </row>
     <row r="180" customFormat="1" spans="1:4">
       <c r="A180">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B180" t="s">
         <v>14</v>
@@ -3625,7 +3618,7 @@
     </row>
     <row r="181" customFormat="1" spans="1:4">
       <c r="A181">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B181" t="s">
         <v>6</v>
@@ -3639,7 +3632,7 @@
     </row>
     <row r="182" customFormat="1" spans="1:4">
       <c r="A182">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B182" t="s">
         <v>14</v>
@@ -3653,7 +3646,7 @@
     </row>
     <row r="183" customFormat="1" spans="1:4">
       <c r="A183">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B183" t="s">
         <v>11</v>
@@ -3667,7 +3660,7 @@
     </row>
     <row r="184" customFormat="1" spans="1:4">
       <c r="A184">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B184" t="s">
         <v>11</v>
@@ -3681,7 +3674,7 @@
     </row>
     <row r="185" customFormat="1" spans="1:4">
       <c r="A185">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B185" t="s">
         <v>11</v>
@@ -3695,7 +3688,7 @@
     </row>
     <row r="186" customFormat="1" spans="1:4">
       <c r="A186">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B186" t="s">
         <v>11</v>
@@ -3709,7 +3702,7 @@
     </row>
     <row r="187" customFormat="1" spans="1:4">
       <c r="A187">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B187" t="s">
         <v>11</v>
@@ -3723,7 +3716,7 @@
     </row>
     <row r="188" customFormat="1" spans="1:4">
       <c r="A188">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B188" t="s">
         <v>11</v>
@@ -3737,7 +3730,7 @@
     </row>
     <row r="189" customFormat="1" spans="1:4">
       <c r="A189">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B189" t="s">
         <v>11</v>
@@ -3751,7 +3744,7 @@
     </row>
     <row r="190" customFormat="1" spans="1:4">
       <c r="A190">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B190" t="s">
         <v>11</v>
@@ -3765,7 +3758,7 @@
     </row>
     <row r="191" customFormat="1" spans="1:4">
       <c r="A191">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B191" t="s">
         <v>14</v>
@@ -3779,7 +3772,7 @@
     </row>
     <row r="192" customFormat="1" spans="1:4">
       <c r="A192">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B192" t="s">
         <v>6</v>
@@ -3793,7 +3786,7 @@
     </row>
     <row r="193" customFormat="1" spans="1:4">
       <c r="A193">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B193" t="s">
         <v>14</v>
@@ -3807,7 +3800,7 @@
     </row>
     <row r="194" customFormat="1" spans="1:4">
       <c r="A194">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B194" t="s">
         <v>6</v>
@@ -3821,7 +3814,7 @@
     </row>
     <row r="195" customFormat="1" spans="1:4">
       <c r="A195">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B195" t="s">
         <v>14</v>
@@ -3835,7 +3828,7 @@
     </row>
     <row r="196" customFormat="1" spans="1:4">
       <c r="A196">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B196" t="s">
         <v>6</v>
@@ -3849,7 +3842,7 @@
     </row>
     <row r="197" customFormat="1" ht="15" customHeight="1" spans="1:4">
       <c r="A197">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B197" t="s">
         <v>14</v>
@@ -3863,7 +3856,7 @@
     </row>
     <row r="198" customFormat="1" spans="1:4">
       <c r="A198">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B198" t="s">
         <v>14</v>
@@ -3877,7 +3870,7 @@
     </row>
     <row r="199" customFormat="1" spans="1:4">
       <c r="A199">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B199" t="s">
         <v>6</v>
@@ -3891,7 +3884,7 @@
     </row>
     <row r="200" customFormat="1" spans="1:4">
       <c r="A200">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B200" t="s">
         <v>14</v>
@@ -3905,7 +3898,7 @@
     </row>
     <row r="201" customFormat="1" spans="1:4">
       <c r="A201">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B201" t="s">
         <v>6</v>
@@ -3919,7 +3912,7 @@
     </row>
     <row r="202" customFormat="1" spans="1:4">
       <c r="A202">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B202" t="s">
         <v>14</v>
@@ -3933,7 +3926,7 @@
     </row>
     <row r="203" customFormat="1" spans="1:4">
       <c r="A203">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B203" t="s">
         <v>6</v>
@@ -3947,7 +3940,7 @@
     </row>
     <row r="204" customFormat="1" spans="1:4">
       <c r="A204">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B204" t="s">
         <v>14</v>
@@ -3961,7 +3954,7 @@
     </row>
     <row r="205" customFormat="1" spans="1:4">
       <c r="A205">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B205" t="s">
         <v>11</v>
@@ -3975,7 +3968,7 @@
     </row>
     <row r="206" customFormat="1" spans="1:4">
       <c r="A206">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B206" t="s">
         <v>11</v>
@@ -3989,7 +3982,7 @@
     </row>
     <row r="207" customFormat="1" spans="1:4">
       <c r="A207">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B207" t="s">
         <v>11</v>
@@ -4003,7 +3996,7 @@
     </row>
     <row r="208" customFormat="1" spans="1:4">
       <c r="A208">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B208" t="s">
         <v>11</v>
@@ -4017,7 +4010,7 @@
     </row>
     <row r="209" customFormat="1" spans="1:4">
       <c r="A209">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B209" t="s">
         <v>11</v>
@@ -4031,7 +4024,7 @@
     </row>
     <row r="210" customFormat="1" spans="1:4">
       <c r="A210">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B210" t="s">
         <v>11</v>
@@ -4045,7 +4038,7 @@
     </row>
     <row r="211" customFormat="1" spans="1:4">
       <c r="A211">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B211" t="s">
         <v>11</v>
@@ -4059,7 +4052,7 @@
     </row>
     <row r="212" customFormat="1" spans="1:4">
       <c r="A212">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B212" t="s">
         <v>11</v>
@@ -4073,7 +4066,7 @@
     </row>
     <row r="213" customFormat="1" spans="1:4">
       <c r="A213">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B213" t="s">
         <v>14</v>
@@ -4087,7 +4080,7 @@
     </row>
     <row r="214" customFormat="1" spans="1:4">
       <c r="A214">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B214" t="s">
         <v>6</v>
@@ -4101,7 +4094,7 @@
     </row>
     <row r="215" customFormat="1" spans="1:4">
       <c r="A215">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B215" t="s">
         <v>14</v>
@@ -4115,7 +4108,7 @@
     </row>
     <row r="216" customFormat="1" spans="1:4">
       <c r="A216">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B216" t="s">
         <v>6</v>
@@ -4129,7 +4122,7 @@
     </row>
     <row r="217" customFormat="1" spans="1:4">
       <c r="A217">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B217" t="s">
         <v>14</v>
@@ -4143,7 +4136,7 @@
     </row>
     <row r="218" customFormat="1" spans="1:4">
       <c r="A218">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B218" t="s">
         <v>6</v>
@@ -4157,7 +4150,7 @@
     </row>
     <row r="219" customFormat="1" ht="15" customHeight="1" spans="1:4">
       <c r="A219">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B219" t="s">
         <v>14</v>
@@ -4171,7 +4164,7 @@
     </row>
     <row r="220" spans="1:4">
       <c r="A220">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B220" t="s">
         <v>15</v>
@@ -4188,7 +4181,7 @@
   <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="B8:F9 B10:F11 C15:F15 B16:F17 A1:F1 C5:F5 B6:F7" numberStoredAsText="1"/>
+    <ignoredError sqref="B6:F11 C15:F15 B16:F17 A1:F1 C5:F5" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>